<commit_message>
feat(api): -Pengujian API via Postman: verifikasi alur Auth (login/logout/me), CRUD master data, proteksi role 403 Forbidden, validasi 422, dan soft deletes berjalan sukses tanpa error. -Memperbarui UserController agar secara otomatis mengosongkan password_hash (set NULL) untuk akun role Kasir.
</commit_message>
<xml_diff>
--- a/Dokumen/Input.xlsx
+++ b/Dokumen/Input.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kuliah\Semester 7\KP\Point-Of-Sale-App\Dokumen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5DF4CD-94FA-4BE3-A069-56B2C52E27BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B647960-0D1E-4AAE-A4FC-19CD168AAEA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2610" yWindow="2595" windowWidth="15375" windowHeight="7875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25725" yWindow="5265" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="65">
   <si>
     <t>Nama Entitas</t>
   </si>
@@ -48,9 +48,6 @@
     <t>Admin</t>
   </si>
   <si>
-    <t>id_user, username, password_hash, nama_user, status_aktif</t>
-  </si>
-  <si>
     <t>Form Registrasi Admin &amp; Kelola Kasir</t>
   </si>
   <si>
@@ -69,9 +66,6 @@
     <t>Kasir &amp; Admin</t>
   </si>
   <si>
-    <t>id_transaksi_detail, harga_produk, quantity, nominal_promo, subtotal_item, status_item, alasan_batal_item</t>
-  </si>
-  <si>
     <t>Halaman Keranjang Belanja APK Mobile</t>
   </si>
   <si>
@@ -93,33 +87,18 @@
     <t>Form Pengaturan Jalur Penjualan</t>
   </si>
   <si>
-    <t>id_template, harga_produk</t>
-  </si>
-  <si>
     <t>Form Sinkronisasi Harga per Cabang</t>
   </si>
   <si>
-    <t>id_kategori, nama_kategori</t>
-  </si>
-  <si>
     <t>Form Manajemen Kategori Produk</t>
   </si>
   <si>
-    <t>id_sub_kategori, nama_sub_kategori</t>
-  </si>
-  <si>
     <t>Form Manajemen Sub Kategori Produk</t>
   </si>
   <si>
-    <t>id_menu, nama_menu</t>
-  </si>
-  <si>
     <t>Form Kelola Master Data Produk</t>
   </si>
   <si>
-    <t>id_promo, nama_promo, tipe_promo, cakupan_promo, nilai_promo, id_menu_free</t>
-  </si>
-  <si>
     <t>Form Input Program Diskon &amp; Promo</t>
   </si>
   <si>
@@ -141,9 +120,6 @@
     <t>RU</t>
   </si>
   <si>
-    <t xml:space="preserve">id_detail_bayar, payment_gateway_id, reference_number, qr_string_data, va_number, status_api </t>
-  </si>
-  <si>
     <t>role_user</t>
   </si>
   <si>
@@ -186,16 +162,64 @@
     <t>promosi</t>
   </si>
   <si>
-    <t>id_cabang, nama_cabang, lokasi,pajak_persen</t>
-  </si>
-  <si>
-    <t>id_shift, waktu_mulai, waktu_selesai, modal_awal, uang_fisik_akhir, status_shift, id_user_aktif, id_cabang, id_sales</t>
-  </si>
-  <si>
-    <t>id_transaksi, tanggal_transaksi, jam_transaksi, nama_pelanggan, tax, total, status, alasan_batal, id_promo, nominal_promo</t>
-  </si>
-  <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>id_kategori, nama_kategori, deleted_at</t>
+  </si>
+  <si>
+    <t>id_user, id_role, id_cabang, username, password_hash, nama_user, status_aktif, deleted_at</t>
+  </si>
+  <si>
+    <t>id_cabang, pajak_persen, nama_cabang, lokasi, deleted_at</t>
+  </si>
+  <si>
+    <t>id_shift, id_user, id_user_aktif, id_cabang, id_sales, waktu_mulai, waktu_selesai, modal_awal, uang_fisik_akhir, status_shift, selisih_uang</t>
+  </si>
+  <si>
+    <t>id_transaksi, id_sales, id_cabang, id_user, id_metode, id_shift, id_promo, tanggal_transaksi, jam_transaksi, nama_pelanggan, tax, total, status, alasan_batal, diperbarui_oleh, catatan_koreksi, nominal_promo</t>
+  </si>
+  <si>
+    <t>id_transaksi_detail, id_transaksi, id_produk, harga_produk, quantity, id_promo, nominal_promo, subtotal_item, status_item, alasan_batal_item</t>
+  </si>
+  <si>
+    <t>id_detail_bayar, id_transaksi, payment_gateway_id, reference_number, qr_string_data, va_number, status_api, waktu_kedaluwarsa, raw_callback_payload</t>
+  </si>
+  <si>
+    <t>id_template, id_menu, id_cabang, id_sales, harga_produk</t>
+  </si>
+  <si>
+    <t>id_sub_kategori, id_kategori, nama_sub_kategori, deleted_at</t>
+  </si>
+  <si>
+    <t>id_menu, id_sub_kategori, nama_menu, deleted_at</t>
+  </si>
+  <si>
+    <t>id_promo, id_cabang, nama_promo, tipe_promo, cakupan_promo, nilai_promo, id_menu_free</t>
+  </si>
+  <si>
+    <t>shift_operator_logs</t>
+  </si>
+  <si>
+    <t>id_log, id_shift, id_user, aksi, waktu_kejadian, catatan</t>
+  </si>
+  <si>
+    <t>Sesi Istirahat &amp; Pergantian Kasir di APK</t>
+  </si>
+  <si>
+    <t>Kasir (Sistem)</t>
+  </si>
+  <si>
+    <t>audit_logs</t>
+  </si>
+  <si>
+    <t>id_audit, id_user, aktivitas, tabel_target, id_target, data_sebelum, data_sesudah, waktu_kejadian, ip_address</t>
+  </si>
+  <si>
+    <t>Log Audit Modifikasi Data Master di Web Admin</t>
+  </si>
+  <si>
+    <t>CR</t>
   </si>
 </sst>
 </file>
@@ -229,7 +253,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -252,11 +276,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -281,6 +333,21 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -502,8 +569,8 @@
   <cols>
     <col min="1" max="1" width="8.7109375" style="2" customWidth="1"/>
     <col min="2" max="2" width="20.5703125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="36.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="29.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="33.140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="22" style="2" customWidth="1"/>
     <col min="6" max="6" width="8.7109375" style="2" customWidth="1"/>
     <col min="7" max="7" width="33.140625" style="2" bestFit="1" customWidth="1"/>
@@ -528,21 +595,21 @@
         <v>3</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I4" s="3" t="s">
         <v>6</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>4</v>
@@ -554,354 +621,406 @@
         <v>6</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>56</v>
+        <v>31</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="J5" s="7" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="6" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>8</v>
       </c>
       <c r="E6" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>35</v>
+        <v>32</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E7" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="H7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" ht="105" x14ac:dyDescent="0.25">
+      <c r="B9" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>56</v>
+      <c r="C9" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>30</v>
       </c>
     </row>
-    <row r="8" spans="2:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D8" s="5" t="s">
+    <row r="10" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="B10" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H8" s="3" t="s">
+      <c r="G10" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="9" spans="2:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" spans="2:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>36</v>
+      <c r="H10" s="1" t="s">
+        <v>29</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B11" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="5" t="s">
+    </row>
+    <row r="12" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G11" s="6" t="s">
+      <c r="G13" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>56</v>
-      </c>
     </row>
-    <row r="12" spans="2:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="B12" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" s="5" t="s">
+    <row r="14" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B14" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B13" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>35</v>
+        <v>40</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B15" s="4" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>25</v>
+        <v>53</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="E15" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="16" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B16" s="4" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>35</v>
+        <v>42</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B17" s="4" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>29</v>
+        <v>54</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>22</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>6</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>35</v>
+        <v>43</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>28</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:10" ht="30" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G18" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="J18" s="7" t="s">
+      <c r="G18" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="I18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>56</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G19" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="I19" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="I20" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
feat: implementasi sinkronisasi batch offline dengan idempotensi serta penambahan modul arsitektur fondasi POS
- Menambahkan dukungan sinkronisasi batch offline dengan prinsip idempotensi pada transaksi dan sesi shift.
- Refaktor dan sinkronisasi presisi skema database (migrations, models, seeders) sesuai spesifikasi Physical Data Model (PDM).
- Memperbarui presisi tipe data DECIMAL(12,2) pada tabel transaksi, transaksi_detail, shift_session, dan menu_template.
- Menyesuaikan batas karakter dan tipe kolom (lokasi ke TEXT NOT NULL di cabang, nama_menu ke VARCHAR(150) di menu).
- Mengembalikan kolom kategori_metode serta menonaktifkan timestamps ($timestamps = false) pada model dan migration metode_pembayaran.
- Memperbarui skema tabel promosi (id_cabang, tipe_promo, cakupan_promo, nilai_promo, id_menu_free) dan seeder terkait.
- Memperbarui relasi dan atribut pada UserModel, StoreUserRequest, UpdateUserRequest, serta password_reset_tokens.
</commit_message>
<xml_diff>
--- a/Dokumen/Input.xlsx
+++ b/Dokumen/Input.xlsx
@@ -603,424 +603,682 @@
       <c r="I4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="3" t="s">
-        <v>26</v>
+      <c r="J4" s="3" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Sistem</x:t>
+        </x:is>
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I5" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="7" t="s">
-        <v>45</v>
+      <c r="B5" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>role_user</x:t>
+        </x:is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_role, nama_role</x:t>
+        </x:is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Web Admin (Sistem)</x:t>
+        </x:is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>role_user</x:t>
+        </x:is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J5" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="6" spans="2:10" ht="60" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="7" t="s">
-        <v>45</v>
+      <c r="B6" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>user</x:t>
+        </x:is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_user, id_role, id_cabang, username, password_hash, nama_user, email, status_aktif, deleted_at</x:t>
+        </x:is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Registrasi Admin &amp; Kelola Kasir</x:t>
+        </x:is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>user</x:t>
+        </x:is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J6" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="7" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="7" t="s">
-        <v>45</v>
+      <c r="B7" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>password_reset_tokens</x:t>
+        </x:is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>email, token, created_at</x:t>
+        </x:is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Lupa Password Web Admin</x:t>
+        </x:is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>password_reset_tokens</x:t>
+        </x:is>
+      </c>
+      <c r="H7" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRU</x:t>
+        </x:is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="8" spans="2:10" ht="75" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>45</v>
+      <c r="B8" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>cabang</x:t>
+        </x:is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_cabang, pajak_persen, nama_cabang, lokasi, deleted_at</x:t>
+        </x:is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Manajemen Cabang</x:t>
+        </x:is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>cabang</x:t>
+        </x:is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J8" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="9" spans="2:10" ht="105" x14ac:dyDescent="0.25">
-      <c r="B9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>30</v>
+      <c r="B9" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>shift_session</x:t>
+        </x:is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_shift, id_user, id_user_aktif, id_cabang, id_sales, waktu_mulai, waktu_selesai, modal_awal, uang_fisik_akhir, status_shift, selisih_uang</x:t>
+        </x:is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Shift (Opening &amp; Closing) di APK</x:t>
+        </x:is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Kasir</x:t>
+        </x:is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>shift_session</x:t>
+        </x:is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRU</x:t>
+        </x:is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="J9" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>U - Auto Close</x:t>
+        </x:is>
       </c>
     </row>
     <row r="10" spans="2:10" ht="75" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>45</v>
+      <c r="B10" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>transaksi</x:t>
+        </x:is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_transaksi, id_sales, id_cabang, id_user, id_metode, id_shift, id_promo, tanggal_transaksi, jam_transaksi, nama_pelanggan, tax, total, status, alasan_batal, diperbarui_oleh, catatan_koreksi, nominal_promo, nomor_referensi</x:t>
+        </x:is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Menu Checkout APK &amp; Koreksi Web Admin</x:t>
+        </x:is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Kasir &amp; Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>transaksi</x:t>
+        </x:is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRU</x:t>
+        </x:is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>RU</x:t>
+        </x:is>
+      </c>
+      <c r="J10" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="11" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B11" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>45</v>
+      <c r="B11" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>transaksi_detail</x:t>
+        </x:is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_transaksi_detail, id_transaksi, id_produk, harga_produk, quantity, id_promo, nominal_promo, subtotal_item, status_item, alasan_batal_item</x:t>
+        </x:is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Halaman Keranjang Belanja APK Mobile</x:t>
+        </x:is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Kasir</x:t>
+        </x:is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>transaksi_detail</x:t>
+        </x:is>
+      </c>
+      <c r="H11" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRU</x:t>
+        </x:is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="12" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B12" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>29</v>
+      <c r="B12" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>shift_operator_logs</x:t>
+        </x:is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_log, id_shift, id_user, aksi, waktu_kejadian, catatan</x:t>
+        </x:is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Sesi Istirahat &amp; Pergantian Kasir di APK</x:t>
+        </x:is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Kasir (Sistem)</x:t>
+        </x:is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>shift_operator_logs</x:t>
+        </x:is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CR</x:t>
+        </x:is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="J12" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="13" spans="2:10" ht="90" x14ac:dyDescent="0.25">
-      <c r="B13" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>45</v>
+      <c r="B13" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>metode_pembayaran</x:t>
+        </x:is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_metode, nama_metode, kategori_metode</x:t>
+        </x:is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Pengaturan Pembayaran</x:t>
+        </x:is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>metode_pembayaran</x:t>
+        </x:is>
+      </c>
+      <c r="H13" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I13" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J13" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="14" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B14" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>45</v>
+      <c r="B14" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>sales_mode</x:t>
+        </x:is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_sales, nama_mode</x:t>
+        </x:is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Pengaturan Jalur Penjualan</x:t>
+        </x:is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>sales_mode</x:t>
+        </x:is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I14" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J14" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="15" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>45</v>
+      <c r="B15" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>menu_template</x:t>
+        </x:is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_template, id_menu, id_cabang, id_sales, harga_produk</x:t>
+        </x:is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Sinkronisasi Harga per Cabang</x:t>
+        </x:is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>menu_template</x:t>
+        </x:is>
+      </c>
+      <c r="H15" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I15" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J15" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="16" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B16" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J16" s="7" t="s">
-        <v>45</v>
+      <c r="B16" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>kategori</x:t>
+        </x:is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_kategori, nama_kategori, deleted_at</x:t>
+        </x:is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Manajemen Kategori Produk</x:t>
+        </x:is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>kategori</x:t>
+        </x:is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I16" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J16" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="17" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B17" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="I17" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>45</v>
+      <c r="B17" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>sub_kategori</x:t>
+        </x:is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_sub_kategori, id_kategori, nama_sub_kategori, deleted_at</x:t>
+        </x:is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Manajemen Sub Kategori Produk</x:t>
+        </x:is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>sub_kategori</x:t>
+        </x:is>
+      </c>
+      <c r="H17" s="1" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J17" s="7" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="18" spans="2:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="B18" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E18" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="I18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J18" s="11" t="s">
-        <v>45</v>
+      <c r="B18" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>menu</x:t>
+        </x:is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_menu, id_sub_kategori, nama_menu, deleted_at</x:t>
+        </x:is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Kelola Master Data Produk</x:t>
+        </x:is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>menu</x:t>
+        </x:is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="19" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="H19" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="I19" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="J19" s="13" t="s">
-        <v>45</v>
+      <c r="B19" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>promosi</x:t>
+        </x:is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_promo, id_cabang, nama_promo, tipe_promo, cakupan_promo, nilai_promo, id_menu_free</x:t>
+        </x:is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Form Input Program Diskon &amp; Promo</x:t>
+        </x:is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>promosi</x:t>
+        </x:is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CRUD</x:t>
+        </x:is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
       </c>
     </row>
     <row r="20" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C20" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G20" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="H20" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="I20" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="J20" s="13" t="s">
-        <v>45</v>
+      <c r="B20" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>audit_logs</x:t>
+        </x:is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>id_audit, id_user, aktivitas, tabel_target, id_target, data_sebelum, data_sesudah, waktu_kejadian, ip_address</x:t>
+        </x:is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Log Audit Modifikasi Data Master di Web Admin</x:t>
+        </x:is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>Admin</x:t>
+        </x:is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>audit_logs</x:t>
+        </x:is>
+      </c>
+      <c r="H20" s="13" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>-</x:t>
+        </x:is>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>R</x:t>
+        </x:is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <x:is xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+          <x:t>CR</x:t>
+        </x:is>
       </c>
     </row>
     <row r="21" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>